<commit_message>
Atualização automática portal mariana
</commit_message>
<xml_diff>
--- a/upload/contabancaria.xlsx
+++ b/upload/contabancaria.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="14">
   <si>
     <t>Ano de Exercício</t>
   </si>
@@ -387,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J190"/>
+  <dimension ref="A1:J199"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -6403,7 +6403,7 @@
         <v>13</v>
       </c>
       <c r="J188">
-        <v>1244405.03</v>
+        <v>8607619.449999999</v>
       </c>
     </row>
     <row r="189" spans="1:10">
@@ -6439,8 +6439,296 @@
       </c>
     </row>
     <row r="190" spans="1:10">
+      <c r="A190">
+        <v>2026</v>
+      </c>
+      <c r="B190">
+        <v>9</v>
+      </c>
+      <c r="C190">
+        <v>9999</v>
+      </c>
+      <c r="D190" t="s">
+        <v>10</v>
+      </c>
+      <c r="E190" t="s">
+        <v>11</v>
+      </c>
+      <c r="F190" t="s">
+        <v>12</v>
+      </c>
+      <c r="G190">
+        <v>9445683</v>
+      </c>
+      <c r="H190">
+        <v>80</v>
+      </c>
+      <c r="I190" t="s">
+        <v>13</v>
+      </c>
       <c r="J190">
-        <v>392362823.26</v>
+        <v>1968287.98</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10">
+      <c r="A191">
+        <v>2026</v>
+      </c>
+      <c r="B191">
+        <v>9</v>
+      </c>
+      <c r="C191">
+        <v>9999</v>
+      </c>
+      <c r="D191" t="s">
+        <v>10</v>
+      </c>
+      <c r="E191" t="s">
+        <v>11</v>
+      </c>
+      <c r="F191" t="s">
+        <v>12</v>
+      </c>
+      <c r="G191">
+        <v>9445684</v>
+      </c>
+      <c r="H191">
+        <v>80</v>
+      </c>
+      <c r="I191" t="s">
+        <v>13</v>
+      </c>
+      <c r="J191">
+        <v>39856.34</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10">
+      <c r="A192">
+        <v>2026</v>
+      </c>
+      <c r="B192">
+        <v>9</v>
+      </c>
+      <c r="C192">
+        <v>9999</v>
+      </c>
+      <c r="D192" t="s">
+        <v>10</v>
+      </c>
+      <c r="E192" t="s">
+        <v>11</v>
+      </c>
+      <c r="F192" t="s">
+        <v>12</v>
+      </c>
+      <c r="G192">
+        <v>9445703</v>
+      </c>
+      <c r="H192">
+        <v>80</v>
+      </c>
+      <c r="I192" t="s">
+        <v>13</v>
+      </c>
+      <c r="J192">
+        <v>390820.04</v>
+      </c>
+    </row>
+    <row r="193" spans="1:10">
+      <c r="A193">
+        <v>2026</v>
+      </c>
+      <c r="B193">
+        <v>9</v>
+      </c>
+      <c r="C193">
+        <v>9999</v>
+      </c>
+      <c r="D193" t="s">
+        <v>10</v>
+      </c>
+      <c r="E193" t="s">
+        <v>11</v>
+      </c>
+      <c r="F193" t="s">
+        <v>12</v>
+      </c>
+      <c r="G193">
+        <v>9445716</v>
+      </c>
+      <c r="H193">
+        <v>80</v>
+      </c>
+      <c r="I193" t="s">
+        <v>13</v>
+      </c>
+      <c r="J193">
+        <v>10682612.8</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10">
+      <c r="A194">
+        <v>2026</v>
+      </c>
+      <c r="B194">
+        <v>9</v>
+      </c>
+      <c r="C194">
+        <v>9999</v>
+      </c>
+      <c r="D194" t="s">
+        <v>10</v>
+      </c>
+      <c r="E194" t="s">
+        <v>11</v>
+      </c>
+      <c r="F194" t="s">
+        <v>12</v>
+      </c>
+      <c r="G194">
+        <v>9445718</v>
+      </c>
+      <c r="H194">
+        <v>80</v>
+      </c>
+      <c r="I194" t="s">
+        <v>13</v>
+      </c>
+      <c r="J194">
+        <v>2762441.83</v>
+      </c>
+    </row>
+    <row r="195" spans="1:10">
+      <c r="A195">
+        <v>2026</v>
+      </c>
+      <c r="B195">
+        <v>9</v>
+      </c>
+      <c r="C195">
+        <v>9999</v>
+      </c>
+      <c r="D195" t="s">
+        <v>10</v>
+      </c>
+      <c r="E195" t="s">
+        <v>11</v>
+      </c>
+      <c r="F195" t="s">
+        <v>12</v>
+      </c>
+      <c r="G195">
+        <v>9445719</v>
+      </c>
+      <c r="H195">
+        <v>80</v>
+      </c>
+      <c r="I195" t="s">
+        <v>13</v>
+      </c>
+      <c r="J195">
+        <v>4410125.01</v>
+      </c>
+    </row>
+    <row r="196" spans="1:10">
+      <c r="A196">
+        <v>2026</v>
+      </c>
+      <c r="B196">
+        <v>9</v>
+      </c>
+      <c r="C196">
+        <v>9999</v>
+      </c>
+      <c r="D196" t="s">
+        <v>10</v>
+      </c>
+      <c r="E196" t="s">
+        <v>11</v>
+      </c>
+      <c r="F196" t="s">
+        <v>12</v>
+      </c>
+      <c r="G196">
+        <v>9445721</v>
+      </c>
+      <c r="H196">
+        <v>80</v>
+      </c>
+      <c r="I196" t="s">
+        <v>13</v>
+      </c>
+      <c r="J196">
+        <v>3260843.18</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10">
+      <c r="A197">
+        <v>2026</v>
+      </c>
+      <c r="B197">
+        <v>9</v>
+      </c>
+      <c r="C197">
+        <v>9999</v>
+      </c>
+      <c r="D197" t="s">
+        <v>10</v>
+      </c>
+      <c r="E197" t="s">
+        <v>11</v>
+      </c>
+      <c r="F197" t="s">
+        <v>12</v>
+      </c>
+      <c r="G197">
+        <v>9445763</v>
+      </c>
+      <c r="H197">
+        <v>80</v>
+      </c>
+      <c r="I197" t="s">
+        <v>13</v>
+      </c>
+      <c r="J197">
+        <v>8608002.51</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10">
+      <c r="A198">
+        <v>2026</v>
+      </c>
+      <c r="B198">
+        <v>9</v>
+      </c>
+      <c r="C198">
+        <v>9999</v>
+      </c>
+      <c r="D198" t="s">
+        <v>10</v>
+      </c>
+      <c r="E198" t="s">
+        <v>11</v>
+      </c>
+      <c r="F198" t="s">
+        <v>12</v>
+      </c>
+      <c r="G198">
+        <v>9447774</v>
+      </c>
+      <c r="H198">
+        <v>80</v>
+      </c>
+      <c r="I198" t="s">
+        <v>13</v>
+      </c>
+      <c r="J198">
+        <v>1506.33</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10">
+      <c r="J199">
+        <v>431850533.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>